<commit_message>
Update sample excel templates with exact headers from word document
</commit_message>
<xml_diff>
--- a/webapp/public/templates/11. THIẾT BỊ PHỤ TRỢ_QUÝ.xlsx
+++ b/webapp/public/templates/11. THIẾT BỊ PHỤ TRỢ_QUÝ.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B7_QUÝ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,58 +413,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Cột 1</t>
+          <t>STT</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Cột 2</t>
+          <t>Trung tâm viễn thông</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Cột 3</t>
+          <t>Số CSHT</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Cột 4</t>
+          <t>Số CSHT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Cột 5</t>
+          <t>Máy nổ</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Cột 6</t>
+          <t>Máy nổ</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Cột 7</t>
+          <t>Máy lạnh</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Cột 8</t>
+          <t>Máy lạnh</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Cột 9</t>
+          <t>Accu</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Cột 10</t>
+          <t>Accu</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Tủ nguồn</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Tủ nguồn</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Tổng thiết bị</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Tổng thiết bị</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bến Lức</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Đức Hòa</t>
         </is>
       </c>
     </row>

</xml_diff>